<commit_message>
feat: add French translation resx files and French README
</commit_message>
<xml_diff>
--- a/ExtremeSkinsTransData.xlsx
+++ b/ExtremeSkinsTransData.xlsx
@@ -1880,975 +1880,975 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr/>
-  </ns0:sheetPr>
-  <ns0:dimension ref="A1:Q80"/>
-  <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
-  <ns0:cols>
-    <ns0:col width="38.368852" customWidth="1" min="1" max="1"/>
-    <ns0:col width="15.245902" customWidth="1" min="2" max="2"/>
-    <ns0:col width="3.631148" customWidth="1" min="3" max="12"/>
-    <ns0:col width="56.245902" customWidth="1" min="13" max="13"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="B1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>English</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Latam</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Brazilian</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Portuguese</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Korean</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Russian</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dutch</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="I1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Filipino</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>French</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>German</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Italian</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Japanese</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Spanish</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>SChinese</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="P1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>TChinese</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="Q1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Irish</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2">
-      <ns0:c r="A2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>kusaZunGreen</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Zunda Green</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>笠ずんちゃん</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O2" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>深墨绿色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3">
-      <ns0:c r="A3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>darkRed</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dark Red</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ダークレッド</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O3" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>深红色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4">
-      <ns0:c r="A4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mediumVioletRed</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Medium Violet Red</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ミディアムバイオレットレッド</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O4" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>紫罗兰红</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5">
-      <ns0:c r="A5" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mediumPurple</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Medium Purple</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M5" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ミディアムパープル</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O5" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>柔和紫</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="6">
-      <ns0:c r="A6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>rosyBrown</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Rose Brown</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ローズブラウン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O6" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>褐玫瑰红</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" t="inlineStr">
-        <ns0:is>
-          <ns0:t>darkMagenta</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B7" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dark Magenta</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M7" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ダークマゼンタ</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O7" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>深洋红色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8">
-      <ns0:c r="A8" t="inlineStr">
-        <ns0:is>
-          <ns0:t>olive</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B8" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Olive</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M8" t="inlineStr">
-        <ns0:is>
-          <ns0:t>オリーブ</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O8" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>橄榄色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="9">
-      <ns0:c r="A9" t="inlineStr">
-        <ns0:is>
-          <ns0:t>steelBlue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B9" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Steel Blue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M9" t="inlineStr">
-        <ns0:is>
-          <ns0:t>スチールブルー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O9" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>钢青色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10">
-      <ns0:c r="A10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dodgerBlue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dodger Blue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ドジャーブルー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O10" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>道奇蓝</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11">
-      <ns0:c r="A11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>darkSeaGreen</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dark Sea Green</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ダークシーグリーン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O11" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>深蓝色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="12">
-      <ns0:c r="A12" t="inlineStr">
-        <ns0:is>
-          <ns0:t>sikon</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B12" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Shikon</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M12" t="inlineStr">
-        <ns0:is>
-          <ns0:t>紫紺</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O12" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>紫青色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="13">
-      <ns0:c r="A13" t="inlineStr">
-        <ns0:is>
-          <ns0:t>konjou</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B13" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Prussian Blue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M13" t="inlineStr">
-        <ns0:is>
-          <ns0:t>紺青</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O13" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>靛蓝色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="A14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>vermilion</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Vermillion</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>バーミリオン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O14" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>朱红色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="15">
-      <ns0:c r="A15" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ivyGreen</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B15" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Ivy Green</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M15" t="inlineStr">
-        <ns0:is>
-          <ns0:t>アイビーグリーン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O15" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>常青藤绿</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16">
-      <ns0:c r="A16" t="inlineStr">
-        <ns0:is>
-          <ns0:t>tilleul</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B16" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Tilleul</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M16" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ティユール</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O16" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>椴树色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="17">
-      <ns0:c r="A17" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ivory</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B17" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Ivory</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M17" t="inlineStr">
-        <ns0:is>
-          <ns0:t>アイボリー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O17" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>象牙色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="18">
-      <ns0:c r="A18" t="inlineStr">
-        <ns0:is>
-          <ns0:t>kenpou</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B18" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Kenpou</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M18" t="inlineStr">
-        <ns0:is>
-          <ns0:t>憲房</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O18" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>深灰色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="19">
-      <ns0:c r="A19" t="inlineStr">
-        <ns0:is>
-          <ns0:t>grisbleu</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B19" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Gris Blue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M19" t="inlineStr">
-        <ns0:is>
-          <ns0:t>グリー・ブルー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O19" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>灰蓝色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="20">
-      <ns0:c r="A20" t="inlineStr">
-        <ns0:is>
-          <ns0:t>melon</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B20" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Melon</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M20" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ムロン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O20" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>柠檬黄</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="21">
-      <ns0:c r="A21" t="inlineStr">
-        <ns0:is>
-          <ns0:t>clan</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B21" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Cranberry</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M21" t="inlineStr">
-        <ns0:is>
-          <ns0:t>クラン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O21" s="6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>浅墨绿色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="22">
-      <ns0:c r="A22" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Shiraaiiro</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B22" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Indigo White</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M22" t="inlineStr">
-        <ns0:is>
-          <ns0:t>白藍</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O22" t="inlineStr">
-        <ns0:is>
-          <ns0:t>靛白色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="23">
-      <ns0:c r="A23" t="inlineStr">
-        <ns0:is>
-          <ns0:t>whitePink</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B23" t="inlineStr">
-        <ns0:is>
-          <ns0:t>White-Pink</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M23" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ホワイトピンク</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O23" t="inlineStr">
-        <ns0:is>
-          <ns0:t>粉白色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="24" ht="21" customHeight="1">
-      <ns0:c r="A24" t="inlineStr">
-        <ns0:is>
-          <ns0:t>thinPurple</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B24" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Thin Purple</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M24" t="inlineStr">
-        <ns0:is>
-          <ns0:t>シンパープル</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O24" t="inlineStr">
-        <ns0:is>
-          <ns0:t>淡紫色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="25">
-      <ns0:c r="A25" t="inlineStr">
-        <ns0:is>
-          <ns0:t>sienna</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B25" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Sienna</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M25" t="inlineStr">
-        <ns0:is>
-          <ns0:t>シエナ</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O25" t="inlineStr">
-        <ns0:is>
-          <ns0:t>土黄色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="26">
-      <ns0:c r="A26" t="inlineStr">
-        <ns0:is>
-          <ns0:t>lightAvocado</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B26" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Light Avocado</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M26" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ライトアヴォーカード</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O26" t="inlineStr">
-        <ns0:is>
-          <ns0:t>淡绿色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="27" ht="20.25" customHeight="1">
-      <ns0:c r="A27" t="inlineStr">
-        <ns0:is>
-          <ns0:t>lightIwaitya</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B27" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Light Iwai-cha</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M27" t="inlineStr">
-        <ns0:is>
-          <ns0:t>薄岩井茶</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O27" t="inlineStr">
-        <ns0:is>
-          <ns0:t>淡褐色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28">
-      <ns0:c r="A28" t="inlineStr">
-        <ns0:is>
-          <ns0:t>diardRed</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B28" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dyad Red</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M28" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ダイアードレッド</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O28" t="inlineStr">
-        <ns0:is>
-          <ns0:t>二红色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="29">
-      <ns0:c r="A29" t="inlineStr">
-        <ns0:is>
-          <ns0:t>diardGreen</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B29" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dyad Green</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M29" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ダイアードグリーン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O29" t="inlineStr">
-        <ns0:is>
-          <ns0:t>二绿色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="30" ht="18.75" customHeight="1">
-      <ns0:c r="A30" t="inlineStr">
-        <ns0:is>
-          <ns0:t>diardBlue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B30" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Dyad Blue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M30" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ダイアードブルー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O30" t="inlineStr">
-        <ns0:is>
-          <ns0:t>二蓝色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="31">
-      <ns0:c r="A31" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chaos</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B31" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Chaos</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M31" t="inlineStr">
-        <ns0:is>
-          <ns0:t>カオス</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O31" t="inlineStr">
-        <ns0:is>
-          <ns0:t>乱色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="32">
-      <ns0:c r="A32" t="inlineStr">
-        <ns0:is>
-          <ns0:t>inverted</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B32" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Inverted</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M32" t="inlineStr">
-        <ns0:is>
-          <ns0:t>インバーテッド</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O32" t="inlineStr">
-        <ns0:is>
-          <ns0:t>反色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="33">
-      <ns0:c r="A33" t="inlineStr">
-        <ns0:is>
-          <ns0:t>oddGreen</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B33" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Odd Green</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M33" t="inlineStr">
-        <ns0:is>
-          <ns0:t>オッドグリーン</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O33" t="inlineStr">
-        <ns0:is>
-          <ns0:t>深绿色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="34">
-      <ns0:c r="A34" t="inlineStr">
-        <ns0:is>
-          <ns0:t>tigr</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B34" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Tiger</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M34" t="inlineStr">
-        <ns0:is>
-          <ns0:t>タイガー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O34" t="inlineStr">
-        <ns0:is>
-          <ns0:t>虎色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="35">
-      <ns0:c r="A35" t="inlineStr">
-        <ns0:is>
-          <ns0:t>kigi</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B35" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Kigi</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M35" t="inlineStr">
-        <ns0:is>
-          <ns0:t>キギ</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O35" t="inlineStr">
-        <ns0:is>
-          <ns0:t>基吉色</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="36">
-      <ns0:c r="A36" t="inlineStr">
-        <ns0:is>
-          <ns0:t>whisky</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B36" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Whisky</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M36" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ウィスキー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="37">
-      <ns0:c r="A37" t="inlineStr">
-        <ns0:is>
-          <ns0:t>geranium</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B37" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Geranium</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M37" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ジェラニョム</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="38">
-      <ns0:c r="A38" t="inlineStr">
-        <ns0:is>
-          <ns0:t>fuchsia</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B38" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Fuchsia</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M38" t="inlineStr">
-        <ns0:is>
-          <ns0:t>フクシャ</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="39">
-      <ns0:c r="A39" t="inlineStr">
-        <ns0:is>
-          <ns0:t>safeBlue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B39" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Safe Blue</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M39" t="inlineStr">
-        <ns0:is>
-          <ns0:t>セーフブルー</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="40"/>
-    <ns0:row r="41"/>
-    <ns0:row r="42"/>
-    <ns0:row r="43"/>
-    <ns0:row r="44"/>
-    <ns0:row r="45"/>
-    <ns0:row r="46"/>
-    <ns0:row r="47"/>
-    <ns0:row r="48"/>
-    <ns0:row r="49"/>
-    <ns0:row r="50"/>
-    <ns0:row r="51" ht="18" customHeight="1"/>
-    <ns0:row r="52" ht="20.25" customHeight="1"/>
-    <ns0:row r="53" ht="19.5" customHeight="1"/>
-    <ns0:row r="54" ht="18.75" customHeight="1"/>
-    <ns0:row r="55">
-      <ns0:c r="M55" s="52" t="n"/>
-    </ns0:row>
-    <ns0:row r="56">
-      <ns0:c r="M56" s="52" t="n"/>
-    </ns0:row>
-    <ns0:row r="57" ht="39" customHeight="1">
-      <ns0:c r="M57" s="52" t="n"/>
-    </ns0:row>
-    <ns0:row r="58">
-      <ns0:c r="M58" s="52" t="n"/>
-    </ns0:row>
-    <ns0:row r="59"/>
-    <ns0:row r="60">
-      <ns0:c r="M60" s="52" t="n"/>
-    </ns0:row>
-    <ns0:row r="61"/>
-    <ns0:row r="62"/>
-    <ns0:row r="63"/>
-    <ns0:row r="64"/>
-    <ns0:row r="65"/>
-    <ns0:row r="66"/>
-    <ns0:row r="67"/>
-    <ns0:row r="68"/>
-    <ns0:row r="69"/>
-    <ns0:row r="70"/>
-    <ns0:row r="71"/>
-    <ns0:row r="72"/>
-    <ns0:row r="73"/>
-    <ns0:row r="74" ht="18.75" customHeight="1"/>
-    <ns0:row r="75" ht="20.25" customHeight="1"/>
-    <ns0:row r="76"/>
-    <ns0:row r="77"/>
-    <ns0:row r="78"/>
-    <ns0:row r="79">
-      <ns0:c r="M79" s="52" t="n"/>
-    </ns0:row>
-    <ns0:row r="80">
-      <ns0:c r="M80" s="52" t="n"/>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ns0:pageSetup paperSize="9" fitToHeight="1" fitToWidth="0"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q80"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
+  <cols>
+    <col width="38.368852" customWidth="1" min="1" max="1"/>
+    <col width="15.245902" customWidth="1" min="2" max="2"/>
+    <col width="3.631148" customWidth="1" min="3" max="12"/>
+    <col width="56.245902" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Latam</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Brazilian</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Portuguese</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Korean</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Russian</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Filipino</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>French</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>German</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Italian</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>SChinese</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>TChinese</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Irish</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>kusaZunGreen</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Zunda Green</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>笠ずんちゃん</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>深墨绿色</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>darkRed</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dark Red</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>ダークレッド</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>深红色</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mediumVioletRed</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Medium Violet Red</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>ミディアムバイオレットレッド</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>紫罗兰红</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mediumPurple</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Medium Purple</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>ミディアムパープル</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>柔和紫</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>rosyBrown</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Rose Brown</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>ローズブラウン</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>褐玫瑰红</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>darkMagenta</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dark Magenta</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>ダークマゼンタ</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>深洋红色</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>olive</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Olive</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>オリーブ</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>橄榄色</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>steelBlue</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Steel Blue</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>スチールブルー</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>钢青色</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dodgerBlue</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dodger Blue</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>ドジャーブルー</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>道奇蓝</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>darkSeaGreen</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dark Sea Green</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>ダークシーグリーン</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>深蓝色</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sikon</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Shikon</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>紫紺</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>紫青色</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>konjou</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Prussian Blue</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>紺青</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>靛蓝色</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>vermilion</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Vermillion</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>バーミリオン</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>朱红色</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ivyGreen</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ivy Green</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>アイビーグリーン</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>常青藤绿</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tilleul</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tilleul</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>ティユール</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>椴树色</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ivory</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ivory</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>アイボリー</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>象牙色</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>kenpou</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Kenpou</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>憲房</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>深灰色</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>grisbleu</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Gris Blue</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>グリー・ブルー</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>灰蓝色</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>melon</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Melon</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>ムロン</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>柠檬黄</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>clan</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cranberry</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>クラン</t>
+        </is>
+      </c>
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>浅墨绿色</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Shiraaiiro</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Indigo White</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>白藍</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>靛白色</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>whitePink</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>White-Pink</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>ホワイトピンク</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>粉白色</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="21" customHeight="1">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>thinPurple</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Thin Purple</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>シンパープル</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>淡紫色</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sienna</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Sienna</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>シエナ</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>土黄色</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>lightAvocado</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Light Avocado</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>ライトアヴォーカード</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>淡绿色</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20.25" customHeight="1">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>lightIwaitya</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Light Iwai-cha</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>薄岩井茶</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>淡褐色</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>diardRed</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Dyad Red</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>ダイアードレッド</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>二红色</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>diardGreen</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Dyad Green</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>ダイアードグリーン</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>二绿色</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18.75" customHeight="1">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>diardBlue</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Dyad Blue</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>ダイアードブルー</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>二蓝色</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>chaos</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Chaos</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>カオス</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>乱色</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>inverted</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Inverted</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>インバーテッド</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>反色</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>oddGreen</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Odd Green</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>オッドグリーン</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>深绿色</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tigr</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Tiger</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>タイガー</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>虎色</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>kigi</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Kigi</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>キギ</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>基吉色</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>whisky</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Whisky</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>ウィスキー</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>geranium</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Geranium</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>ジェラニョム</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>fuchsia</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Fuchsia</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>フクシャ</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>safeBlue</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Safe Blue</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>セーフブルー</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51" ht="18" customHeight="1"/>
+    <row r="52" ht="20.25" customHeight="1"/>
+    <row r="53" ht="19.5" customHeight="1"/>
+    <row r="54" ht="18.75" customHeight="1"/>
+    <row r="55">
+      <c r="M55" s="52" t="n"/>
+    </row>
+    <row r="56">
+      <c r="M56" s="52" t="n"/>
+    </row>
+    <row r="57" ht="39" customHeight="1">
+      <c r="M57" s="52" t="n"/>
+    </row>
+    <row r="58">
+      <c r="M58" s="52" t="n"/>
+    </row>
+    <row r="59"/>
+    <row r="60">
+      <c r="M60" s="52" t="n"/>
+    </row>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74" ht="18.75" customHeight="1"/>
+    <row r="75" ht="20.25" customHeight="1"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79">
+      <c r="M79" s="52" t="n"/>
+    </row>
+    <row r="80">
+      <c r="M80" s="52" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToHeight="1" fitToWidth="0"/>
+</worksheet>
 </file>
</xml_diff>